<commit_message>
Add store-visit-date and POSM photo filename columns to Bridgestone import template
Visit Date already tracked which day a store was completed; adds paired
filename columns for signage/POSM/cube/counter-flyer photos so the client
can reference per-store, per-channel POSM pictures sent alongside the sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/reports/bridgestone/bridgestone-mystery-shopper-import-template.xlsx
+++ b/public/reports/bridgestone/bridgestone-mystery-shopper-import-template.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -447,24 +447,28 @@
     <col width="46" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
     <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="30" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="22" customWidth="1" min="29" max="29"/>
-    <col width="40" customWidth="1" min="30" max="30"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="33" max="33"/>
+    <col width="40" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -530,90 +534,110 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Signage Photo Filename</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Bridgestone POSM Available</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Firestone POSM Available</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Type of POSM Present</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>POSM Photo Filename</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Bridgestone POSM Cube Visible</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>POSM Cube Photo Filename</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Bridgestone POSM Counter Flyer Visible</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Counter Flyer Photo Filename</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Brand Recommended by Staff</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Tyre SKU Recommended</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Bridgestone Stock Available</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Firestone Stock Available</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Warranty Offered</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Warranty Details</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Promotion Mentioned</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recommendation Basis (Price/Quality)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Competitor Brand Mentioned</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Discovery Questions Asked</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Time Spent With Customer (mins)</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Consultant / Staff Name</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Notable Quote / Comments</t>
         </is>
@@ -682,88 +706,108 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>BRG-0001_signage.jpg</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Fixed Tyre Stand, Posters</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>BRG-0001_posm.jpg</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>BRG-0001_cube.jpg</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>BRG-0001_flyer.jpg</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>Bridgestone</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Bridgestone Dueler AT002</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>Bridgestone Firestone 1 Year</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AB2" t="n">
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
         <v>12</v>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>J. Adams</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>"They walked me through the tread pattern before quoting."</t>
         </is>
@@ -832,7 +876,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>BRG-0002_signage.jpg</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -842,78 +886,98 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>Till Brochures, Counter Flyer</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>BRG-0002_posm.jpg</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>BRG-0002_cube.jpg</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>BRG-0002_flyer.jpg</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>Bridgestone</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Bridgestone T005</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Dunlop Sure</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AB3" t="n">
+      <c r="AF3" t="n">
         <v>6</v>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>T. Naidoo</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="17">
@@ -935,37 +999,37 @@
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="V2:V1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
     <dataValidation sqref="X2:X1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="Y2:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
     <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AB2:AB1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD2:AD1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE2:AE1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Price,Quality"</formula1>
     </dataValidation>
   </dataValidations>
@@ -979,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1038,9 +1102,43 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Send the completed file back to Leegra for import into the dashboard and live in-app questionnaire history.</t>
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Uploading POSM photos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Name each photo file starting with the Store Code, e.g. BRG-0001_signage.jpg, BRG-0001_posm.jpg, BRG-0001_cube.jpg, BRG-0001_flyer.jpg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Put the exact filename in the matching column (Signage Photo Filename / POSM Photo Filename / POSM Cube Photo Filename / Counter Flyer Photo Filename) on that store's row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Send the actual photo files back to Leegra together with this spreadsheet (a folder or zip is fine) — the spreadsheet only tells us which photo belongs to which store and question, it doesn't carry the image itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Send the completed file (and photos) back to Leegra for import into the dashboard and live in-app questionnaire history.</t>
         </is>
       </c>
     </row>

</xml_diff>